<commit_message>
[Comp-753] Report tweaks (#836)
</commit_message>
<xml_diff>
--- a/compliance-api/src/compliance_api/services/report/first_nation_template.xlsx
+++ b/compliance-api/src/compliance_api/services/report/first_nation_template.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
-  <workbookPr hidePivotFieldList="1"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tayalee/Desktop/Excel pivot tables_forfeedback/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E89B9424-7BF0-434C-8C25-63EDBB9A2830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{95A6700E-82FC-4D1E-A6B4-B1AE8DE46F72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="35080" yWindow="1540" windowWidth="34560" windowHeight="20260" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inspections" sheetId="13" r:id="rId1"/>
-    <sheet name="InsightsInsights" sheetId="3" r:id="rId2"/>
+    <sheet name="InspectionInsights" sheetId="3" r:id="rId2"/>
     <sheet name="Complaints" sheetId="14" r:id="rId3"/>
     <sheet name="ComplaintsInsights" sheetId="15" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191028"/>
   <pivotCaches>
-    <pivotCache cacheId="386" r:id="rId5"/>
-    <pivotCache cacheId="381" r:id="rId6"/>
+    <pivotCache cacheId="1850" r:id="rId5"/>
+    <pivotCache cacheId="1859" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="30">
   <si>
     <t>IR Number</t>
   </si>
@@ -101,6 +101,12 @@
     <t>Attended Inspections</t>
   </si>
   <si>
+    <t>Count of First Nation/First Nation Alliance</t>
+  </si>
+  <si>
+    <t>Column Labels</t>
+  </si>
+  <si>
     <t>Row Labels</t>
   </si>
   <si>
@@ -143,13 +149,10 @@
     <t>Complaint Specifics and Outcomes by Project</t>
   </si>
   <si>
-    <t>Complaint Tpoics by Project</t>
+    <t>Complaint Topics by Project</t>
   </si>
   <si>
     <t>Count of Complaint Number</t>
-  </si>
-  <si>
-    <t>Column Labels</t>
   </si>
   <si>
     <t>(All)</t>
@@ -175,7 +178,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -185,6 +188,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -232,20 +241,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="3"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="16">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -262,14 +264,18 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="none"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -308,7 +314,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor theme="3"/>
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
     </dxf>
@@ -328,14 +343,26 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.39997558519241921"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="none"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.39997558519241921"/>
+        </patternFill>
       </fill>
     </dxf>
   </dxfs>
@@ -352,74 +379,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46149.453074305558" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{489B308B-C5F1-4496-9EA3-999C745CB76D}">
-  <cacheSource type="worksheet">
-    <worksheetSource name="Complaints"/>
-  </cacheSource>
-  <cacheFields count="12">
-    <cacheField name="Complaint Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Complaint Source" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Complaint Source Details" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Project Name" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Project Type" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Topic" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Concern Description" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Date Received" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Primary Officer" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Complaint Status" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Complaint Resolution" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
-        <m/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Case File Number" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46149.453074305558" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2E3C93A3-DEF7-49F3-8ED9-11D95FDFFC7E}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46155.585315856479" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{2E3C93A3-DEF7-49F3-8ED9-11D95FDFFC7E}">
   <cacheSource type="worksheet">
     <worksheetSource name="Inspections"/>
   </cacheSource>
@@ -430,7 +390,9 @@
       </sharedItems>
     </cacheField>
     <cacheField name="First Nation/First Nation Alliance" numFmtId="0">
-      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
     </cacheField>
     <cacheField name="IR Progress" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
@@ -448,7 +410,7 @@
         <m/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Inspetion End Date" numFmtId="0">
+    <cacheField name="Inspection End Date" numFmtId="0">
       <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="IR Issuance Date" numFmtId="0">
@@ -469,9 +431,72 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" saveData="0" refreshOnLoad="1" refreshedBy="Excel Services" refreshedDate="46155.585315856479" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="1" xr:uid="{489B308B-C5F1-4496-9EA3-999C745CB76D}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Complaints"/>
+  </cacheSource>
+  <cacheFields count="12">
+    <cacheField name="Complaint Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Complaint Source" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Complaint Source Details" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Name" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Project Type" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Topic" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Concern Description" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Date Received" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Primary Officer" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Complaint Status" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Complaint Resolution" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1" count="1">
+        <m/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Case File Number" numFmtId="0">
+      <sharedItems containsNonDate="0" containsString="0" containsBlank="1"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{99612004-EEE9-4DAE-800E-65B87BD035A0}" name="Attended Inspections" cacheId="381" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B4:B8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{99612004-EEE9-4DAE-800E-65B87BD035A0}" name="Attended Inspections" cacheId="1850" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B4:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField axis="axisRow" showAll="0">
       <items count="2">
@@ -479,7 +504,12 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="2">
@@ -518,23 +548,34 @@
       <x/>
     </i>
   </rowItems>
-  <colItems count="1">
-    <i/>
+  <colFields count="1">
+    <field x="1"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
   </colItems>
+  <dataFields count="1">
+    <dataField name="Count of First Nation/First Nation Alliance" fld="1" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
   <formats count="5">
-    <format dxfId="10">
+    <format dxfId="11">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="11">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="12">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="13">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea field="5" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
     <format dxfId="14">
+      <pivotArea field="1" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
+    </format>
+    <format dxfId="15">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -551,7 +592,107 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A78A3DE9-337B-4375-ABAF-39D54018E350}" name="Complaint Specifics and Outcomes by Project" cacheId="386" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DC00558-9D6A-4D8C-A8BC-4CABB5BCD879}" name="Complaint Topics by Project" cacheId="1859" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="I6:J10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="2">
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="2"/>
+    <field x="3"/>
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="9" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Complaint Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="7">
+    <format dxfId="4">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="5">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="6">
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="7">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="8">
+      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+    </format>
+    <format dxfId="9">
+      <pivotArea field="2" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
+    </format>
+    <format dxfId="10">
+      <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A78A3DE9-337B-4375-ABAF-39D54018E350}" name="Complaint Specifics and Outcomes by Project" cacheId="1859" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B4:D9" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -620,124 +761,17 @@
   <dataFields count="1">
     <dataField name="Count of Complaint Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
-  <formats count="5">
-    <format dxfId="5">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="6">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="7">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="8">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="9">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4DC00558-9D6A-4D8C-A8BC-4CABB5BCD879}" name="Complaint Topics by Project" cacheId="386" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="I6:J10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="2">
-        <item sd="0" x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="2">
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="3">
-    <field x="2"/>
-    <field x="3"/>
-    <field x="5"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="2">
-      <x/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="9" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Complaint Number" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="5">
+  <formats count="4">
     <format dxfId="0">
       <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="1">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
     <format dxfId="2">
-      <pivotArea type="origin" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
+      <pivotArea field="10" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisCol" fieldPosition="0"/>
     </format>
     <format dxfId="3">
-      <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
-    </format>
-    <format dxfId="4">
       <pivotArea type="topRight" dataOnly="0" labelOnly="1" outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -1134,10 +1168,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C3DA8C2-D460-3E49-93A1-0DC80ABEB419}">
-  <dimension ref="B2:B8"/>
+  <dimension ref="B2:D9"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.7109375" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
@@ -1219,35 +1253,58 @@
     <col min="124" max="124" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:4">
       <c r="B2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="2:2">
-      <c r="B4" s="1" t="s">
+    <row r="4" spans="2:4">
+      <c r="B4" s="4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="2:2">
-      <c r="B5" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="2:2">
-      <c r="B6" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2">
-      <c r="B7" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2">
-      <c r="B8" s="2" t="s">
+      <c r="D4" s="4"/>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="B5" s="7" t="s">
         <v>13</v>
       </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="B6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="B7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="B8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
@@ -1276,37 +1333,37 @@
   <sheetData>
     <row r="1" spans="1:12">
       <c r="A1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E1" t="s">
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="L1" s="6" t="s">
         <v>9</v>
@@ -1328,8 +1385,12 @@
     <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="6" max="6" width="25.85546875" customWidth="1"/>
+    <col min="7" max="7" width="23.42578125" customWidth="1"/>
+    <col min="8" max="8" width="26.5703125" customWidth="1"/>
     <col min="9" max="9" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="29" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -1338,89 +1399,89 @@
   <sheetData>
     <row r="2" spans="2:10">
       <c r="B2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="2:10">
       <c r="B4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="8"/>
+        <v>28</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="4"/>
       <c r="I4" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="2:10">
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="2:10">
       <c r="B6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="I6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>26</v>
+        <v>14</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="I6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="2:10">
       <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
       <c r="I7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J7" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="J7" s="8"/>
     </row>
     <row r="8" spans="2:10">
       <c r="B8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
       <c r="I8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="J8" s="8"/>
     </row>
     <row r="9" spans="2:10">
       <c r="B9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
       <c r="I9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="J9" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="J9" s="8"/>
     </row>
     <row r="10" spans="2:10">
       <c r="I10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J10" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="J10" s="8"/>
     </row>
     <row r="11" spans="2:10">
       <c r="B11" s="2"/>

</xml_diff>